<commit_message>
chore: remove AutoMapper e corrige DTOs quebrados do dashboard
- Remove AutoMapper (vulnerabilidade de seguranca alta, GHSA-rvv3-g6hj-g44x)
  dos projetos Application, Infrastructure e App; mapeamento manual via
  novo ProjetoDtoMapper em CriarProjetoUseCase, EditarProjetoUseCase e
  ListarProjetosUseCase.
- Corrige referencias quebradas a DTOs renomeados (DashboardDTO,
  AtividadeResponseDTO) e reescreve DashboardService para o novo formato
  (ProjetoRecenteDTO, IndicadorCriticidadeDTO); AtividadesAtrasadas fica
  vazio ate o redesenho de dominio decidir como resolver ProjetoNome/
  ResponsavelNome em Atividade.
- Adiciona harness Claude (.claude/, .specs/, CLAUDE.md) e padroes de
  design system vendorizados (Docs/Padroes_CygnusForge/).
- Atualiza assets visuais para o rebranding do produto para FlowForge.
</commit_message>
<xml_diff>
--- a/Docs/Definições.xlsx
+++ b/Docs/Definições.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcos.Araujo\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marcos\source\repos\CygnusFlow\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5769EC-4C8D-46D9-9106-BF01C78CED67}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C787220E-F1DE-4B55-84CA-6AAA75173FA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13590" windowHeight="6705" activeTab="1" xr2:uid="{6A9CE72F-87A5-4853-AECB-BDC6A8BF55EA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6A9CE72F-87A5-4853-AECB-BDC6A8BF55EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Critérios" sheetId="1" r:id="rId1"/>
     <sheet name="Cenarios Testes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="DadosExternos_1" localSheetId="1" hidden="1">'Cenarios Testes'!$A$1:$E$24</definedName>
+    <definedName name="DadosExternos_1" localSheetId="1" hidden="1">'Cenarios Testes'!$A$1:$E$28</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="180">
   <si>
     <t>Quando</t>
   </si>
@@ -576,12 +576,54 @@
   <si>
     <t>Pode filtrar por : Equipe, Perfil, Status</t>
   </si>
+  <si>
+    <t>Pode incluir/remover links externos</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Vinculo por registro</t>
+  </si>
+  <si>
+    <t>Adicionado em um projeto</t>
+  </si>
+  <si>
+    <t>Não deve influenciar outros registros que tenham o mesmo link</t>
+  </si>
+  <si>
+    <t>Link Externo vinculado no projeto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projeto </t>
+  </si>
+  <si>
+    <t>Link Externo excluído no projeto</t>
+  </si>
+  <si>
+    <t>Exclusão de vinculo por registro</t>
+  </si>
+  <si>
+    <t>Removido de um projeto</t>
+  </si>
+  <si>
+    <t>Link Externo vinculado na atividade</t>
+  </si>
+  <si>
+    <t>Link Externo excluído na atividade</t>
+  </si>
+  <si>
+    <t>Adicionado em uma atividade</t>
+  </si>
+  <si>
+    <t>Removido de uma atividade</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,6 +660,13 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -639,7 +688,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -657,6 +706,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -691,8 +746,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C5D6C1F-FF1D-4724-94E4-408F9353E686}" name="CygnusFlow_Criterios_Cenarios_Teste" displayName="CygnusFlow_Criterios_Cenarios_Teste" ref="A1:E24" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:E24" xr:uid="{D1511B47-1D94-4E5A-B0DD-41BA1A091229}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C5D6C1F-FF1D-4724-94E4-408F9353E686}" name="CygnusFlow_Criterios_Cenarios_Teste" displayName="CygnusFlow_Criterios_Cenarios_Teste" ref="A1:E28" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:E28" xr:uid="{D1511B47-1D94-4E5A-B0DD-41BA1A091229}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{CB5EAA40-D7BB-4226-AFA3-40D0B998298E}" uniqueName="1" name="Módulo" queryTableFieldId="1"/>
     <tableColumn id="2" xr3:uid="{BB6BBC22-220F-469B-9565-9CD3B8B5CA5A}" uniqueName="2" name="Critério" queryTableFieldId="2"/>
@@ -705,9 +760,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -745,7 +800,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -851,7 +906,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -993,7 +1048,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1002,19 +1057,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA96F8D-B30F-4BE3-829F-CEAA475F72B8}">
   <dimension ref="A1:D93"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" style="1" customWidth="1"/>
     <col min="2" max="2" width="19" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="109.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="45.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="109.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
       <c r="C1" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="15.75">
+    <row r="3" spans="1:4" ht="15.6">
       <c r="B3" s="1" t="s">
         <v>31</v>
       </c>
@@ -1431,7 +1486,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="15.75">
+    <row r="46" spans="1:4" ht="15.6">
       <c r="C46" s="3"/>
     </row>
     <row r="48" spans="1:4">
@@ -1490,8 +1545,19 @@
         <v>131</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="15.75">
-      <c r="C52" s="3"/>
+    <row r="52" spans="1:4" ht="15.6">
+      <c r="A52" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="6" t="s">
@@ -1535,7 +1601,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="15.75">
+    <row r="57" spans="1:4" ht="15.6">
       <c r="C57" s="3"/>
     </row>
     <row r="59" spans="1:4">
@@ -1600,7 +1666,7 @@
       </c>
       <c r="D65"/>
     </row>
-    <row r="66" spans="1:4" ht="15.75">
+    <row r="66" spans="1:4" ht="15.6">
       <c r="C66" s="3"/>
       <c r="D66"/>
     </row>
@@ -1693,10 +1759,20 @@
       </c>
     </row>
     <row r="74" spans="1:4">
-      <c r="C74"/>
-      <c r="D74"/>
-    </row>
-    <row r="75" spans="1:4" ht="15.75">
+      <c r="A74" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15.6">
       <c r="C75" s="3"/>
       <c r="D75"/>
     </row>
@@ -1775,10 +1851,20 @@
       </c>
     </row>
     <row r="82" spans="1:4">
-      <c r="C82"/>
-      <c r="D82"/>
-    </row>
-    <row r="83" spans="1:4" ht="15.75">
+      <c r="A82" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="15.6">
       <c r="C83" s="3"/>
       <c r="D83"/>
     </row>
@@ -1832,7 +1918,7 @@
       <c r="C88"/>
       <c r="D88"/>
     </row>
-    <row r="89" spans="1:4" ht="15.75">
+    <row r="89" spans="1:4" ht="15.6">
       <c r="C89" s="3"/>
       <c r="D89"/>
     </row>
@@ -1890,14 +1976,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84B9E01D-BFB8-44B2-9439-B38B6D48418E}">
-  <dimension ref="A1:E24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2140,36 +2226,36 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>172</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>171</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>168</v>
       </c>
       <c r="D15" t="s">
-        <v>70</v>
+        <v>169</v>
       </c>
       <c r="E15" t="s">
-        <v>65</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>172</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>173</v>
       </c>
       <c r="C16" t="s">
-        <v>92</v>
+        <v>174</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2177,16 +2263,16 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -2194,117 +2280,185 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="D18" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>14</v>
       </c>
       <c r="D20" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>176</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>168</v>
       </c>
       <c r="D21" t="s">
-        <v>17</v>
+        <v>178</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>177</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>174</v>
       </c>
       <c r="D22" t="s">
-        <v>22</v>
+        <v>179</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E23" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
+        <v>50</v>
+      </c>
+      <c r="D24" t="s">
+        <v>18</v>
+      </c>
+      <c r="E24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" t="s">
+        <v>71</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
         <v>20</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D26" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" t="s">
         <v>26</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C28" t="s">
         <v>27</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D28" t="s">
         <v>81</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E28" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>